<commit_message>
large file handling,integration and indexing
</commit_message>
<xml_diff>
--- a/pandas/dataFiles/sales.xlsx
+++ b/pandas/dataFiles/sales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
   <si>
     <t>id</t>
   </si>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t>Tablet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id </t>
   </si>
 </sst>
 </file>
@@ -432,7 +429,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>

</xml_diff>